<commit_message>
Atualizar resultados Censo ES Tempo Integral
</commit_message>
<xml_diff>
--- a/outputs/tabelas/es_af_tempo_integral_2015_2025.xlsx
+++ b/outputs/tabelas/es_af_tempo_integral_2015_2025.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R11"/>
+  <dimension ref="A1:V11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,67 +444,87 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>escolas_estaduais_com_af_integral_25pct</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>escolas_municipais_com_af</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>escolas_municipais_com_af_integral</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>matriculas_publicas_af</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>matriculas_publicas_af_integral</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>matriculas_estaduais_af</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>matriculas_estaduais_af_integral</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>matriculas_municipais_af</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>matriculas_municipais_af_integral</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>pct_escolas_publicas_af_integral</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>pct_escolas_estaduais_af_integral</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>pct_escolas_estaduais_af_integral_25pct</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
         <is>
           <t>pct_escolas_municipais_af_integral</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>pct_matriculas_estaduais_af_integral</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>pct_matriculas_municipais_af_integral</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>var_liquida_escolas_estaduais_af_integral</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>var_liquida_matriculas_estaduais_af_integral</t>
         </is>
       </c>
     </row>
@@ -525,44 +545,52 @@
         <v>114</v>
       </c>
       <c r="F2" t="n">
+        <v>39</v>
+      </c>
+      <c r="G2" t="n">
         <v>552</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>301</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>193598</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>22468</v>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>69733</v>
       </c>
-      <c r="K2" t="n">
+      <c r="L2" t="n">
         <v>4225</v>
       </c>
-      <c r="L2" t="n">
+      <c r="M2" t="n">
         <v>123865</v>
       </c>
-      <c r="M2" t="n">
+      <c r="N2" t="n">
         <v>18243</v>
       </c>
-      <c r="N2" t="n">
+      <c r="O2" t="n">
         <v>49.1</v>
       </c>
-      <c r="O2" t="n">
+      <c r="P2" t="n">
         <v>38.8</v>
       </c>
-      <c r="P2" t="n">
+      <c r="Q2" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="R2" t="n">
         <v>54.5</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="S2" t="n">
         <v>6.1</v>
       </c>
-      <c r="R2" t="n">
+      <c r="T2" t="n">
         <v>14.7</v>
       </c>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -581,43 +609,55 @@
         <v>25</v>
       </c>
       <c r="F3" t="n">
+        <v>18</v>
+      </c>
+      <c r="G3" t="n">
         <v>548</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>158</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>193033</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>10927</v>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>69576</v>
       </c>
-      <c r="K3" t="n">
+      <c r="L3" t="n">
         <v>1963</v>
       </c>
-      <c r="L3" t="n">
+      <c r="M3" t="n">
         <v>123457</v>
       </c>
-      <c r="M3" t="n">
+      <c r="N3" t="n">
         <v>8964</v>
       </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
         <v>21.9</v>
       </c>
-      <c r="O3" t="n">
+      <c r="P3" t="n">
         <v>8.699999999999999</v>
       </c>
-      <c r="P3" t="n">
+      <c r="Q3" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="R3" t="n">
         <v>28.8</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="S3" t="n">
         <v>2.8</v>
       </c>
-      <c r="R3" t="n">
+      <c r="T3" t="n">
         <v>7.3</v>
+      </c>
+      <c r="U3" t="n">
+        <v>-89</v>
+      </c>
+      <c r="V3" t="n">
+        <v>-2262</v>
       </c>
     </row>
     <row r="4">
@@ -637,43 +677,55 @@
         <v>29</v>
       </c>
       <c r="F4" t="n">
+        <v>25</v>
+      </c>
+      <c r="G4" t="n">
         <v>548</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>163</v>
       </c>
-      <c r="H4" t="n">
+      <c r="I4" t="n">
         <v>194176</v>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
         <v>12557</v>
       </c>
-      <c r="J4" t="n">
+      <c r="K4" t="n">
         <v>70357</v>
       </c>
-      <c r="K4" t="n">
+      <c r="L4" t="n">
         <v>3455</v>
       </c>
-      <c r="L4" t="n">
+      <c r="M4" t="n">
         <v>123819</v>
       </c>
-      <c r="M4" t="n">
+      <c r="N4" t="n">
         <v>9102</v>
       </c>
-      <c r="N4" t="n">
+      <c r="O4" t="n">
         <v>22.9</v>
       </c>
-      <c r="O4" t="n">
+      <c r="P4" t="n">
         <v>10</v>
       </c>
-      <c r="P4" t="n">
+      <c r="Q4" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="R4" t="n">
         <v>29.7</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="S4" t="n">
         <v>4.9</v>
       </c>
-      <c r="R4" t="n">
+      <c r="T4" t="n">
         <v>7.4</v>
+      </c>
+      <c r="U4" t="n">
+        <v>4</v>
+      </c>
+      <c r="V4" t="n">
+        <v>1492</v>
       </c>
     </row>
     <row r="5">
@@ -693,43 +745,55 @@
         <v>40</v>
       </c>
       <c r="F5" t="n">
+        <v>31</v>
+      </c>
+      <c r="G5" t="n">
         <v>542</v>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>100</v>
       </c>
-      <c r="H5" t="n">
+      <c r="I5" t="n">
         <v>195268</v>
       </c>
-      <c r="I5" t="n">
+      <c r="J5" t="n">
         <v>9354</v>
       </c>
-      <c r="J5" t="n">
+      <c r="K5" t="n">
         <v>72719</v>
       </c>
-      <c r="K5" t="n">
+      <c r="L5" t="n">
         <v>4749</v>
       </c>
-      <c r="L5" t="n">
+      <c r="M5" t="n">
         <v>122549</v>
       </c>
-      <c r="M5" t="n">
+      <c r="N5" t="n">
         <v>4605</v>
       </c>
-      <c r="N5" t="n">
+      <c r="O5" t="n">
         <v>17</v>
       </c>
-      <c r="O5" t="n">
+      <c r="P5" t="n">
         <v>14.1</v>
       </c>
-      <c r="P5" t="n">
+      <c r="Q5" t="n">
+        <v>11</v>
+      </c>
+      <c r="R5" t="n">
         <v>18.5</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="S5" t="n">
         <v>6.5</v>
       </c>
-      <c r="R5" t="n">
+      <c r="T5" t="n">
         <v>3.8</v>
+      </c>
+      <c r="U5" t="n">
+        <v>11</v>
+      </c>
+      <c r="V5" t="n">
+        <v>1294</v>
       </c>
     </row>
     <row r="6">
@@ -749,43 +813,55 @@
         <v>42</v>
       </c>
       <c r="F6" t="n">
+        <v>36</v>
+      </c>
+      <c r="G6" t="n">
         <v>530</v>
       </c>
-      <c r="G6" t="n">
+      <c r="H6" t="n">
         <v>132</v>
       </c>
-      <c r="H6" t="n">
+      <c r="I6" t="n">
         <v>194515</v>
       </c>
-      <c r="I6" t="n">
+      <c r="J6" t="n">
         <v>11711</v>
       </c>
-      <c r="J6" t="n">
+      <c r="K6" t="n">
         <v>75582</v>
       </c>
-      <c r="K6" t="n">
+      <c r="L6" t="n">
         <v>5103</v>
       </c>
-      <c r="L6" t="n">
+      <c r="M6" t="n">
         <v>118933</v>
       </c>
-      <c r="M6" t="n">
+      <c r="N6" t="n">
         <v>6608</v>
       </c>
-      <c r="N6" t="n">
+      <c r="O6" t="n">
         <v>21.3</v>
       </c>
-      <c r="O6" t="n">
+      <c r="P6" t="n">
         <v>14.7</v>
       </c>
-      <c r="P6" t="n">
+      <c r="Q6" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="R6" t="n">
         <v>24.9</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="S6" t="n">
         <v>6.8</v>
       </c>
-      <c r="R6" t="n">
+      <c r="T6" t="n">
         <v>5.6</v>
+      </c>
+      <c r="U6" t="n">
+        <v>2</v>
+      </c>
+      <c r="V6" t="n">
+        <v>354</v>
       </c>
     </row>
     <row r="7">
@@ -805,43 +881,55 @@
         <v>59</v>
       </c>
       <c r="F7" t="n">
+        <v>54</v>
+      </c>
+      <c r="G7" t="n">
         <v>530</v>
       </c>
-      <c r="G7" t="n">
+      <c r="H7" t="n">
         <v>90</v>
       </c>
-      <c r="H7" t="n">
+      <c r="I7" t="n">
         <v>193607</v>
       </c>
-      <c r="I7" t="n">
+      <c r="J7" t="n">
         <v>14392</v>
       </c>
-      <c r="J7" t="n">
+      <c r="K7" t="n">
         <v>75121</v>
       </c>
-      <c r="K7" t="n">
+      <c r="L7" t="n">
         <v>9800</v>
       </c>
-      <c r="L7" t="n">
+      <c r="M7" t="n">
         <v>118486</v>
       </c>
-      <c r="M7" t="n">
+      <c r="N7" t="n">
         <v>4592</v>
       </c>
-      <c r="N7" t="n">
+      <c r="O7" t="n">
         <v>18.1</v>
       </c>
-      <c r="O7" t="n">
+      <c r="P7" t="n">
         <v>20.2</v>
       </c>
-      <c r="P7" t="n">
+      <c r="Q7" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="R7" t="n">
         <v>17</v>
       </c>
-      <c r="Q7" t="n">
+      <c r="S7" t="n">
         <v>13</v>
       </c>
-      <c r="R7" t="n">
+      <c r="T7" t="n">
         <v>3.9</v>
+      </c>
+      <c r="U7" t="n">
+        <v>17</v>
+      </c>
+      <c r="V7" t="n">
+        <v>4697</v>
       </c>
     </row>
     <row r="8">
@@ -861,43 +949,55 @@
         <v>75</v>
       </c>
       <c r="F8" t="n">
+        <v>70</v>
+      </c>
+      <c r="G8" t="n">
         <v>530</v>
       </c>
-      <c r="G8" t="n">
+      <c r="H8" t="n">
         <v>85</v>
       </c>
-      <c r="H8" t="n">
+      <c r="I8" t="n">
         <v>197286</v>
       </c>
-      <c r="I8" t="n">
+      <c r="J8" t="n">
         <v>21364</v>
       </c>
-      <c r="J8" t="n">
+      <c r="K8" t="n">
         <v>75559</v>
       </c>
-      <c r="K8" t="n">
+      <c r="L8" t="n">
         <v>13893</v>
       </c>
-      <c r="L8" t="n">
+      <c r="M8" t="n">
         <v>121727</v>
       </c>
-      <c r="M8" t="n">
+      <c r="N8" t="n">
         <v>7471</v>
       </c>
-      <c r="N8" t="n">
+      <c r="O8" t="n">
         <v>19.4</v>
       </c>
-      <c r="O8" t="n">
+      <c r="P8" t="n">
         <v>25.6</v>
       </c>
-      <c r="P8" t="n">
+      <c r="Q8" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="R8" t="n">
         <v>16</v>
       </c>
-      <c r="Q8" t="n">
+      <c r="S8" t="n">
         <v>18.4</v>
       </c>
-      <c r="R8" t="n">
+      <c r="T8" t="n">
         <v>6.1</v>
+      </c>
+      <c r="U8" t="n">
+        <v>16</v>
+      </c>
+      <c r="V8" t="n">
+        <v>4093</v>
       </c>
     </row>
     <row r="9">
@@ -917,43 +1017,55 @@
         <v>118</v>
       </c>
       <c r="F9" t="n">
+        <v>88</v>
+      </c>
+      <c r="G9" t="n">
         <v>536</v>
       </c>
-      <c r="G9" t="n">
+      <c r="H9" t="n">
         <v>196</v>
       </c>
-      <c r="H9" t="n">
+      <c r="I9" t="n">
         <v>192093</v>
       </c>
-      <c r="I9" t="n">
+      <c r="J9" t="n">
         <v>29391</v>
       </c>
-      <c r="J9" t="n">
+      <c r="K9" t="n">
         <v>71509</v>
       </c>
-      <c r="K9" t="n">
+      <c r="L9" t="n">
         <v>18605</v>
       </c>
-      <c r="L9" t="n">
+      <c r="M9" t="n">
         <v>120584</v>
       </c>
-      <c r="M9" t="n">
+      <c r="N9" t="n">
         <v>10786</v>
       </c>
-      <c r="N9" t="n">
+      <c r="O9" t="n">
         <v>38.1</v>
       </c>
-      <c r="O9" t="n">
+      <c r="P9" t="n">
         <v>41</v>
       </c>
-      <c r="P9" t="n">
+      <c r="Q9" t="n">
+        <v>30.6</v>
+      </c>
+      <c r="R9" t="n">
         <v>36.6</v>
       </c>
-      <c r="Q9" t="n">
+      <c r="S9" t="n">
         <v>26</v>
       </c>
-      <c r="R9" t="n">
+      <c r="T9" t="n">
         <v>8.9</v>
+      </c>
+      <c r="U9" t="n">
+        <v>43</v>
+      </c>
+      <c r="V9" t="n">
+        <v>4712</v>
       </c>
     </row>
     <row r="10">
@@ -973,43 +1085,55 @@
         <v>131</v>
       </c>
       <c r="F10" t="n">
+        <v>103</v>
+      </c>
+      <c r="G10" t="n">
         <v>532</v>
       </c>
-      <c r="G10" t="n">
+      <c r="H10" t="n">
         <v>176</v>
       </c>
-      <c r="H10" t="n">
+      <c r="I10" t="n">
         <v>188872</v>
       </c>
-      <c r="I10" t="n">
+      <c r="J10" t="n">
         <v>31817</v>
       </c>
-      <c r="J10" t="n">
+      <c r="K10" t="n">
         <v>67993</v>
       </c>
-      <c r="K10" t="n">
+      <c r="L10" t="n">
         <v>21358</v>
       </c>
-      <c r="L10" t="n">
+      <c r="M10" t="n">
         <v>120879</v>
       </c>
-      <c r="M10" t="n">
+      <c r="N10" t="n">
         <v>10459</v>
       </c>
-      <c r="N10" t="n">
+      <c r="O10" t="n">
         <v>37.7</v>
       </c>
-      <c r="O10" t="n">
+      <c r="P10" t="n">
         <v>46.5</v>
       </c>
-      <c r="P10" t="n">
+      <c r="Q10" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="R10" t="n">
         <v>33.1</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="S10" t="n">
         <v>31.4</v>
       </c>
-      <c r="R10" t="n">
+      <c r="T10" t="n">
         <v>8.699999999999999</v>
+      </c>
+      <c r="U10" t="n">
+        <v>13</v>
+      </c>
+      <c r="V10" t="n">
+        <v>2753</v>
       </c>
     </row>
     <row r="11">
@@ -1029,43 +1153,55 @@
         <v>126</v>
       </c>
       <c r="F11" t="n">
+        <v>117</v>
+      </c>
+      <c r="G11" t="n">
         <v>535</v>
       </c>
-      <c r="G11" t="n">
+      <c r="H11" t="n">
         <v>185</v>
       </c>
-      <c r="H11" t="n">
+      <c r="I11" t="n">
         <v>185840</v>
       </c>
-      <c r="I11" t="n">
+      <c r="J11" t="n">
         <v>35297</v>
       </c>
-      <c r="J11" t="n">
+      <c r="K11" t="n">
         <v>61106</v>
       </c>
-      <c r="K11" t="n">
+      <c r="L11" t="n">
         <v>23666</v>
       </c>
-      <c r="L11" t="n">
+      <c r="M11" t="n">
         <v>124734</v>
       </c>
-      <c r="M11" t="n">
+      <c r="N11" t="n">
         <v>11631</v>
       </c>
-      <c r="N11" t="n">
+      <c r="O11" t="n">
         <v>38.9</v>
       </c>
-      <c r="O11" t="n">
+      <c r="P11" t="n">
         <v>47.5</v>
       </c>
-      <c r="P11" t="n">
+      <c r="Q11" t="n">
+        <v>44.2</v>
+      </c>
+      <c r="R11" t="n">
         <v>34.6</v>
       </c>
-      <c r="Q11" t="n">
+      <c r="S11" t="n">
         <v>38.7</v>
       </c>
-      <c r="R11" t="n">
+      <c r="T11" t="n">
         <v>9.300000000000001</v>
+      </c>
+      <c r="U11" t="n">
+        <v>-5</v>
+      </c>
+      <c r="V11" t="n">
+        <v>2308</v>
       </c>
     </row>
   </sheetData>

</xml_diff>